<commit_message>
test: update live run reports
</commit_message>
<xml_diff>
--- a/Testing/TEST_RESULTS.xlsx
+++ b/Testing/TEST_RESULTS.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:09.920Z</t>
+          <t>2026-02-25T15:17:06.056Z</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-02-25T15:10:13.500Z</t>
+          <t>2026-02-25T15:19:06.748Z</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>123.58 seconds</t>
+          <t>120.69 seconds</t>
         </is>
       </c>
     </row>
@@ -762,11 +762,11 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:14.136Z</t>
+          <t>2026-02-25T15:17:11.003Z</t>
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>3748</v>
+        <v>8476</v>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
@@ -793,11 +793,11 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:17.884Z</t>
+          <t>2026-02-25T15:17:19.480Z</t>
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>1014</v>
+        <v>758</v>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -824,11 +824,11 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:18.898Z</t>
+          <t>2026-02-25T15:17:20.239Z</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>1833</v>
+        <v>1784</v>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
@@ -855,11 +855,11 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:20.732Z</t>
+          <t>2026-02-25T15:17:22.023Z</t>
         </is>
       </c>
       <c r="E7" s="9" t="n">
-        <v>3024</v>
+        <v>2813</v>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
@@ -886,11 +886,11 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:23.756Z</t>
+          <t>2026-02-25T15:17:24.837Z</t>
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
@@ -917,11 +917,11 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:24.110Z</t>
+          <t>2026-02-25T15:17:25.202Z</t>
         </is>
       </c>
       <c r="E9" s="9" t="n">
-        <v>2923</v>
+        <v>2970</v>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
@@ -948,11 +948,11 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:27.033Z</t>
+          <t>2026-02-25T15:17:28.172Z</t>
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>2949</v>
+        <v>2913</v>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
@@ -979,11 +979,11 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:29.983Z</t>
+          <t>2026-02-25T15:17:31.085Z</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>3055</v>
+        <v>2870</v>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
@@ -1010,11 +1010,11 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:33.041Z</t>
+          <t>2026-02-25T15:17:33.955Z</t>
         </is>
       </c>
       <c r="E12" s="9" t="n">
-        <v>2978</v>
+        <v>1903</v>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
@@ -1041,11 +1041,11 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:36.022Z</t>
+          <t>2026-02-25T15:17:35.858Z</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
-        <v>4703</v>
+        <v>3641</v>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
@@ -1072,11 +1072,11 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:40.726Z</t>
+          <t>2026-02-25T15:17:39.499Z</t>
         </is>
       </c>
       <c r="E14" s="9" t="n">
-        <v>323</v>
+        <v>167</v>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
@@ -1103,11 +1103,11 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:41.050Z</t>
+          <t>2026-02-25T15:17:39.667Z</t>
         </is>
       </c>
       <c r="E15" s="9" t="n">
-        <v>2373</v>
+        <v>1814</v>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
@@ -1134,11 +1134,11 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:43.423Z</t>
+          <t>2026-02-25T15:17:41.494Z</t>
         </is>
       </c>
       <c r="E16" s="9" t="n">
-        <v>3931</v>
+        <v>2911</v>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
@@ -1165,11 +1165,11 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:47.354Z</t>
+          <t>2026-02-25T15:17:44.405Z</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>395</v>
+        <v>335</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
@@ -1196,11 +1196,11 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:47.750Z</t>
+          <t>2026-02-25T15:17:44.741Z</t>
         </is>
       </c>
       <c r="E18" s="9" t="n">
-        <v>12084</v>
+        <v>10262</v>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
@@ -1227,11 +1227,11 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:08:59.835Z</t>
+          <t>2026-02-25T15:17:55.004Z</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
-        <v>3746</v>
+        <v>3126</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
@@ -1258,11 +1258,11 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:03.581Z</t>
+          <t>2026-02-25T15:17:58.131Z</t>
         </is>
       </c>
       <c r="E20" s="9" t="n">
-        <v>1728</v>
+        <v>1718</v>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
@@ -1289,11 +1289,11 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:05.309Z</t>
+          <t>2026-02-25T15:17:59.849Z</t>
         </is>
       </c>
       <c r="E21" s="9" t="n">
-        <v>2565</v>
+        <v>2673</v>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
@@ -1320,11 +1320,11 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:07.874Z</t>
+          <t>2026-02-25T15:18:02.522Z</t>
         </is>
       </c>
       <c r="E22" s="9" t="n">
-        <v>353</v>
+        <v>336</v>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
@@ -1351,11 +1351,11 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:08.228Z</t>
+          <t>2026-02-25T15:18:02.858Z</t>
         </is>
       </c>
       <c r="E23" s="9" t="n">
-        <v>10936</v>
+        <v>10469</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
@@ -1382,11 +1382,11 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:19.164Z</t>
+          <t>2026-02-25T15:18:13.327Z</t>
         </is>
       </c>
       <c r="E24" s="9" t="n">
-        <v>3733</v>
+        <v>3117</v>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
@@ -1413,11 +1413,11 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:22.898Z</t>
+          <t>2026-02-25T15:18:16.444Z</t>
         </is>
       </c>
       <c r="E25" s="9" t="n">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
@@ -1444,11 +1444,11 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:23.027Z</t>
+          <t>2026-02-25T15:18:16.546Z</t>
         </is>
       </c>
       <c r="E26" s="9" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
@@ -1475,11 +1475,11 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:23.047Z</t>
+          <t>2026-02-25T15:18:16.558Z</t>
         </is>
       </c>
       <c r="E27" s="9" t="n">
-        <v>3548</v>
+        <v>3349</v>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
@@ -1506,11 +1506,11 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:31.550Z</t>
+          <t>2026-02-25T15:18:24.803Z</t>
         </is>
       </c>
       <c r="E28" s="9" t="n">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
@@ -1537,11 +1537,11 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:32.137Z</t>
+          <t>2026-02-25T15:18:25.394Z</t>
         </is>
       </c>
       <c r="E29" s="9" t="n">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
@@ -1568,11 +1568,11 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:32.678Z</t>
+          <t>2026-02-25T15:18:25.934Z</t>
         </is>
       </c>
       <c r="E30" s="9" t="n">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
@@ -1599,11 +1599,11 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:33.222Z</t>
+          <t>2026-02-25T15:18:26.474Z</t>
         </is>
       </c>
       <c r="E31" s="9" t="n">
-        <v>1737</v>
+        <v>1686</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -1630,11 +1630,11 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:34.959Z</t>
+          <t>2026-02-25T15:18:28.160Z</t>
         </is>
       </c>
       <c r="E32" s="9" t="n">
-        <v>888</v>
+        <v>794</v>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
@@ -1661,11 +1661,11 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:35.847Z</t>
+          <t>2026-02-25T15:18:28.954Z</t>
         </is>
       </c>
       <c r="E33" s="9" t="n">
-        <v>877</v>
+        <v>822</v>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
@@ -1692,11 +1692,11 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:36.725Z</t>
+          <t>2026-02-25T15:18:29.777Z</t>
         </is>
       </c>
       <c r="E34" s="9" t="n">
-        <v>780</v>
+        <v>765</v>
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
@@ -1723,11 +1723,11 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:37.505Z</t>
+          <t>2026-02-25T15:18:30.542Z</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
-        <v>3127</v>
+        <v>2672</v>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
@@ -1754,11 +1754,11 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:40.632Z</t>
+          <t>2026-02-25T15:18:33.215Z</t>
         </is>
       </c>
       <c r="E36" s="9" t="n">
-        <v>3896</v>
+        <v>3603</v>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
@@ -1785,11 +1785,11 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:44.529Z</t>
+          <t>2026-02-25T15:18:36.822Z</t>
         </is>
       </c>
       <c r="E37" s="9" t="n">
-        <v>468</v>
+        <v>478</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:44.997Z</t>
+          <t>2026-02-25T15:18:37.301Z</t>
         </is>
       </c>
       <c r="E38" s="9" t="n">
@@ -1847,11 +1847,11 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:45.451Z</t>
+          <t>2026-02-25T15:18:37.755Z</t>
         </is>
       </c>
       <c r="E39" s="9" t="n">
-        <v>461</v>
+        <v>442</v>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
@@ -1878,11 +1878,11 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:45.912Z</t>
+          <t>2026-02-25T15:18:38.197Z</t>
         </is>
       </c>
       <c r="E40" s="9" t="n">
-        <v>939</v>
+        <v>778</v>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
@@ -1909,11 +1909,11 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:47.593Z</t>
+          <t>2026-02-25T15:18:39.947Z</t>
         </is>
       </c>
       <c r="E41" s="9" t="n">
-        <v>5438</v>
+        <v>5700</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
@@ -1940,11 +1940,11 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:53.032Z</t>
+          <t>2026-02-25T15:18:45.651Z</t>
         </is>
       </c>
       <c r="E42" s="9" t="n">
-        <v>5971</v>
+        <v>6530</v>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
@@ -1971,11 +1971,11 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:09:59.004Z</t>
+          <t>2026-02-25T15:18:52.185Z</t>
         </is>
       </c>
       <c r="E43" s="9" t="n">
-        <v>2192</v>
+        <v>2204</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
@@ -2002,11 +2002,11 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:10:01.197Z</t>
+          <t>2026-02-25T15:18:54.389Z</t>
         </is>
       </c>
       <c r="E44" s="9" t="n">
-        <v>337</v>
+        <v>350</v>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
@@ -2033,11 +2033,11 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:10:01.534Z</t>
+          <t>2026-02-25T15:18:54.739Z</t>
         </is>
       </c>
       <c r="E45" s="9" t="n">
-        <v>2390</v>
+        <v>2399</v>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
@@ -2064,11 +2064,11 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:10:03.925Z</t>
+          <t>2026-02-25T15:18:57.139Z</t>
         </is>
       </c>
       <c r="E46" s="9" t="n">
-        <v>1393</v>
+        <v>1383</v>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
@@ -2095,11 +2095,11 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:10:05.318Z</t>
+          <t>2026-02-25T15:18:58.523Z</t>
         </is>
       </c>
       <c r="E47" s="9" t="n">
-        <v>4617</v>
+        <v>4741</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
@@ -2126,11 +2126,11 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:10:09.935Z</t>
+          <t>2026-02-25T15:19:03.264Z</t>
         </is>
       </c>
       <c r="E48" s="9" t="n">
-        <v>1764</v>
+        <v>1863</v>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
@@ -2157,11 +2157,11 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:10:11.699Z</t>
+          <t>2026-02-25T15:19:05.127Z</t>
         </is>
       </c>
       <c r="E49" s="9" t="n">
-        <v>497</v>
+        <v>437</v>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
test: stabilize T39 persistence check and update live reports
</commit_message>
<xml_diff>
--- a/Testing/TEST_RESULTS.xlsx
+++ b/Testing/TEST_RESULTS.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:06.056Z</t>
+          <t>2026-02-26T14:37:59.458Z</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-02-25T15:19:06.748Z</t>
+          <t>2026-02-26T14:39:41.680Z</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>120.69 seconds</t>
+          <t>102.22 seconds</t>
         </is>
       </c>
     </row>
@@ -762,11 +762,11 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:11.003Z</t>
+          <t>2026-02-26T14:38:01.407Z</t>
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>8476</v>
+        <v>2109</v>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
@@ -793,11 +793,11 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:19.480Z</t>
+          <t>2026-02-26T14:38:03.516Z</t>
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>758</v>
+        <v>704</v>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -824,11 +824,11 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:20.239Z</t>
+          <t>2026-02-26T14:38:04.220Z</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>1784</v>
+        <v>1679</v>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
@@ -855,11 +855,11 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:22.023Z</t>
+          <t>2026-02-26T14:38:05.900Z</t>
         </is>
       </c>
       <c r="E7" s="9" t="n">
-        <v>2813</v>
+        <v>2446</v>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
@@ -886,11 +886,11 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:24.837Z</t>
+          <t>2026-02-26T14:38:08.347Z</t>
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>364</v>
+        <v>294</v>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
@@ -917,11 +917,11 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:25.202Z</t>
+          <t>2026-02-26T14:38:08.642Z</t>
         </is>
       </c>
       <c r="E9" s="9" t="n">
-        <v>2970</v>
+        <v>2675</v>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
@@ -948,11 +948,11 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:28.172Z</t>
+          <t>2026-02-26T14:38:11.318Z</t>
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>2913</v>
+        <v>2768</v>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
@@ -979,11 +979,11 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:31.085Z</t>
+          <t>2026-02-26T14:38:14.086Z</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>2870</v>
+        <v>2628</v>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
@@ -1010,11 +1010,11 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:33.955Z</t>
+          <t>2026-02-26T14:38:16.715Z</t>
         </is>
       </c>
       <c r="E12" s="9" t="n">
-        <v>1903</v>
+        <v>1829</v>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
@@ -1041,11 +1041,11 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:35.858Z</t>
+          <t>2026-02-26T14:38:18.545Z</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
-        <v>3641</v>
+        <v>2903</v>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
@@ -1072,11 +1072,11 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:39.499Z</t>
+          <t>2026-02-26T14:38:21.449Z</t>
         </is>
       </c>
       <c r="E14" s="9" t="n">
-        <v>167</v>
+        <v>91</v>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
@@ -1103,11 +1103,11 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:39.667Z</t>
+          <t>2026-02-26T14:38:21.541Z</t>
         </is>
       </c>
       <c r="E15" s="9" t="n">
-        <v>1814</v>
+        <v>1697</v>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
@@ -1134,11 +1134,11 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:41.494Z</t>
+          <t>2026-02-26T14:38:23.238Z</t>
         </is>
       </c>
       <c r="E16" s="9" t="n">
-        <v>2911</v>
+        <v>2352</v>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
@@ -1165,11 +1165,11 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:44.405Z</t>
+          <t>2026-02-26T14:38:25.590Z</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>335</v>
+        <v>311</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
@@ -1196,11 +1196,11 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:44.741Z</t>
+          <t>2026-02-26T14:38:25.902Z</t>
         </is>
       </c>
       <c r="E18" s="9" t="n">
-        <v>10262</v>
+        <v>10400</v>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
@@ -1227,11 +1227,11 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:55.004Z</t>
+          <t>2026-02-26T14:38:36.302Z</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
-        <v>3126</v>
+        <v>3263</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
@@ -1258,11 +1258,11 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:58.131Z</t>
+          <t>2026-02-26T14:38:39.566Z</t>
         </is>
       </c>
       <c r="E20" s="9" t="n">
-        <v>1718</v>
+        <v>1742</v>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
@@ -1289,11 +1289,11 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:17:59.849Z</t>
+          <t>2026-02-26T14:38:41.309Z</t>
         </is>
       </c>
       <c r="E21" s="9" t="n">
-        <v>2673</v>
+        <v>2532</v>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
@@ -1320,11 +1320,11 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:02.522Z</t>
+          <t>2026-02-26T14:38:43.842Z</t>
         </is>
       </c>
       <c r="E22" s="9" t="n">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
@@ -1351,11 +1351,11 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:02.858Z</t>
+          <t>2026-02-26T14:38:44.183Z</t>
         </is>
       </c>
       <c r="E23" s="9" t="n">
-        <v>10469</v>
+        <v>10281</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
@@ -1382,11 +1382,11 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:13.327Z</t>
+          <t>2026-02-26T14:38:54.464Z</t>
         </is>
       </c>
       <c r="E24" s="9" t="n">
-        <v>3117</v>
+        <v>3032</v>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
@@ -1413,11 +1413,11 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:16.444Z</t>
+          <t>2026-02-26T14:38:57.496Z</t>
         </is>
       </c>
       <c r="E25" s="9" t="n">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
@@ -1444,11 +1444,11 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:16.546Z</t>
+          <t>2026-02-26T14:38:57.582Z</t>
         </is>
       </c>
       <c r="E26" s="9" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
@@ -1475,11 +1475,11 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:16.558Z</t>
+          <t>2026-02-26T14:38:57.597Z</t>
         </is>
       </c>
       <c r="E27" s="9" t="n">
-        <v>3349</v>
+        <v>3410</v>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
@@ -1506,11 +1506,11 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:24.803Z</t>
+          <t>2026-02-26T14:39:03.951Z</t>
         </is>
       </c>
       <c r="E28" s="9" t="n">
-        <v>591</v>
+        <v>573</v>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
@@ -1537,11 +1537,11 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:25.394Z</t>
+          <t>2026-02-26T14:39:04.525Z</t>
         </is>
       </c>
       <c r="E29" s="9" t="n">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
@@ -1568,11 +1568,11 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:25.934Z</t>
+          <t>2026-02-26T14:39:05.071Z</t>
         </is>
       </c>
       <c r="E30" s="9" t="n">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
@@ -1599,11 +1599,11 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:26.474Z</t>
+          <t>2026-02-26T14:39:05.607Z</t>
         </is>
       </c>
       <c r="E31" s="9" t="n">
-        <v>1686</v>
+        <v>1738</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -1630,11 +1630,11 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:28.160Z</t>
+          <t>2026-02-26T14:39:07.348Z</t>
         </is>
       </c>
       <c r="E32" s="9" t="n">
-        <v>794</v>
+        <v>861</v>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
@@ -1661,11 +1661,11 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:28.954Z</t>
+          <t>2026-02-26T14:39:08.210Z</t>
         </is>
       </c>
       <c r="E33" s="9" t="n">
-        <v>822</v>
+        <v>800</v>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
@@ -1692,11 +1692,11 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:29.777Z</t>
+          <t>2026-02-26T14:39:09.010Z</t>
         </is>
       </c>
       <c r="E34" s="9" t="n">
-        <v>765</v>
+        <v>816</v>
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
@@ -1723,11 +1723,11 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:30.542Z</t>
+          <t>2026-02-26T14:39:09.826Z</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
-        <v>2672</v>
+        <v>2643</v>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
@@ -1754,11 +1754,11 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:33.215Z</t>
+          <t>2026-02-26T14:39:12.469Z</t>
         </is>
       </c>
       <c r="E36" s="9" t="n">
-        <v>3603</v>
+        <v>3422</v>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
@@ -1785,11 +1785,11 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:36.822Z</t>
+          <t>2026-02-26T14:39:15.892Z</t>
         </is>
       </c>
       <c r="E37" s="9" t="n">
-        <v>478</v>
+        <v>451</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
@@ -1816,11 +1816,11 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:37.301Z</t>
+          <t>2026-02-26T14:39:16.343Z</t>
         </is>
       </c>
       <c r="E38" s="9" t="n">
-        <v>454</v>
+        <v>441</v>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
@@ -1847,11 +1847,11 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:37.755Z</t>
+          <t>2026-02-26T14:39:16.785Z</t>
         </is>
       </c>
       <c r="E39" s="9" t="n">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
@@ -1878,11 +1878,11 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:38.197Z</t>
+          <t>2026-02-26T14:39:17.229Z</t>
         </is>
       </c>
       <c r="E40" s="9" t="n">
-        <v>778</v>
+        <v>821</v>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
@@ -1909,11 +1909,11 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:39.947Z</t>
+          <t>2026-02-26T14:39:18.501Z</t>
         </is>
       </c>
       <c r="E41" s="9" t="n">
-        <v>5700</v>
+        <v>4788</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
@@ -1940,11 +1940,11 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:45.651Z</t>
+          <t>2026-02-26T14:39:23.289Z</t>
         </is>
       </c>
       <c r="E42" s="9" t="n">
-        <v>6530</v>
+        <v>5488</v>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
@@ -1971,11 +1971,11 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:52.185Z</t>
+          <t>2026-02-26T14:39:28.777Z</t>
         </is>
       </c>
       <c r="E43" s="9" t="n">
-        <v>2204</v>
+        <v>2012</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
@@ -2002,11 +2002,11 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:54.389Z</t>
+          <t>2026-02-26T14:39:30.790Z</t>
         </is>
       </c>
       <c r="E44" s="9" t="n">
-        <v>350</v>
+        <v>372</v>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
@@ -2033,11 +2033,11 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:54.739Z</t>
+          <t>2026-02-26T14:39:31.162Z</t>
         </is>
       </c>
       <c r="E45" s="9" t="n">
-        <v>2399</v>
+        <v>2389</v>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
@@ -2064,11 +2064,11 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:57.139Z</t>
+          <t>2026-02-26T14:39:33.551Z</t>
         </is>
       </c>
       <c r="E46" s="9" t="n">
-        <v>1383</v>
+        <v>1377</v>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
@@ -2095,11 +2095,11 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:18:58.523Z</t>
+          <t>2026-02-26T14:39:34.928Z</t>
         </is>
       </c>
       <c r="E47" s="9" t="n">
-        <v>4741</v>
+        <v>4691</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
@@ -2126,11 +2126,11 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:19:03.264Z</t>
+          <t>2026-02-26T14:39:39.619Z</t>
         </is>
       </c>
       <c r="E48" s="9" t="n">
-        <v>1863</v>
+        <v>1521</v>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
@@ -2157,11 +2157,11 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>2026-02-25T15:19:05.127Z</t>
+          <t>2026-02-26T14:39:41.140Z</t>
         </is>
       </c>
       <c r="E49" s="9" t="n">
-        <v>437</v>
+        <v>185</v>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
update live run reports
</commit_message>
<xml_diff>
--- a/Testing/TEST_RESULTS.xlsx
+++ b/Testing/TEST_RESULTS.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-02T10:17:26.251Z</t>
+          <t>2026-03-02T11:24:09.324Z</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-03-02T10:17:29.171Z</t>
+          <t>2026-03-02T11:26:15.806Z</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2.92 seconds</t>
+          <t>126.48 seconds</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
@@ -618,17 +618,17 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -639,17 +639,17 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -660,17 +660,17 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -747,33 +747,1428 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Login Admin (GUI)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:10.802Z</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>3364</v>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Open Admin Panel</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:14.166Z</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>695</v>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Create Admin user</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:14.861Z</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>1696</v>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Login nuovo Admin</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:16.557Z</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>3280</v>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Logout Admin-test</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:19.838Z</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>308</v>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Disable Admin-test</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:20.146Z</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>3339</v>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Login utente disabilitato</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:23.486Z</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>2755</v>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Riattivazione Admin-test</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:26.242Z</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>3269</v>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Login post-riattivazione</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:29.511Z</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>2426</v>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Delete Admin-test</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:31.938Z</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>3556</v>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Verify DB clean (API)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:35.494Z</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>689</v>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Create Trader user</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:36.183Z</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>4118</v>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Login Trader</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:40.301Z</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>3068</v>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Logout Trader</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:43.370Z</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>289</v>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Disable/Enable Trader cycle</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:43.660Z</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>11954</v>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Delete Trader</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:55.615Z</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>3765</v>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Create Viewer user</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:24:59.381Z</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>1687</v>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>T18</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Login Viewer</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:01.068Z</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>3215</v>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>T19</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Logout Viewer</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:04.284Z</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>309</v>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Disable/Enable Viewer cycle</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:04.593Z</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>12214</v>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Delete Viewer</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:16.807Z</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>4659</v>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Verify DB clean (API)</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:21.466Z</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>791</v>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Verify GUI clean</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:22.258Z</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>2993</v>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Create users for Section 2</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:25.251Z</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>3413</v>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>T25</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Drag &amp; Drop column</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:32.011Z</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>553</v>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>T26</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Hide column</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:32.565Z</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>534</v>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>T27</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Show column</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:33.100Z</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>535</v>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>T28</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Reset All Columns</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:33.636Z</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>T29</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Sort ascending</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:35.336Z</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>897</v>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>T30</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Sort descending</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:36.233Z</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>879</v>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>T31</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Sort different column</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:37.112Z</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>937</v>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>T32</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Persist country tab after logout</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:38.050Z</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>6306</v>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>T33</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Persist sort after logout</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:44.357Z</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>3737</v>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>T34</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Single filter</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:48.094Z</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>454</v>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>T35</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Multiple filters</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:48.548Z</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>435</v>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>T36</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Remove one filter</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:48.984Z</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>434</v>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>T37</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Clear all filters</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:49.418Z</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>815</v>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>T38</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Mixed modifications</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:50.234Z</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>5711</v>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>T39</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Persist all after reload</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:25:55.945Z</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="n">
+        <v>6188</v>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>T40</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Complete reset</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:26:02.133Z</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>2040</v>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>T42</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Login admin for RFQ tests</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:26:04.174Z</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>359</v>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>T43</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Double-click bond row opens RFQ window</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:26:04.533Z</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>2366</v>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>T44</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>RFQ window displays pricing data</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:26:06.900Z</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>1364</v>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>T45</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>RFQ window draggable and closable</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:26:08.264Z</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>4873</v>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>T46</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Open RFQ from OPEN RFQ button</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:26:13.137Z</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="n">
+        <v>1670</v>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
           <t>T47</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>Final cleanup</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>GUI</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>2026-03-02T10:17:27.665Z</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="n">
-        <v>828</v>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="n"/>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>GUI</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>2026-03-02T11:26:14.807Z</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>556</v>
+      </c>
+      <c r="F49" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Harden live E2E script and refresh reports
</commit_message>
<xml_diff>
--- a/Testing/TEST_RESULTS.xlsx
+++ b/Testing/TEST_RESULTS.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-03-02T15:10:55.212Z</t>
+          <t>2026-03-03T15:47:54.944Z</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-03-02T15:13:15.693Z</t>
+          <t>2026-03-03T15:51:18.023Z</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>140.48 seconds</t>
+          <t>203.08 seconds</t>
         </is>
       </c>
     </row>
@@ -762,11 +762,11 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:10:58.571Z</t>
+          <t>2026-03-03T15:47:57.696Z</t>
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>7284</v>
+        <v>5382</v>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
@@ -793,11 +793,11 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:05.856Z</t>
+          <t>2026-03-03T15:48:03.078Z</t>
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>1190</v>
+        <v>734</v>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -824,11 +824,11 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:07.046Z</t>
+          <t>2026-03-03T15:48:03.812Z</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>1928</v>
+        <v>1736</v>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
@@ -855,11 +855,11 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:08.975Z</t>
+          <t>2026-03-03T15:48:05.548Z</t>
         </is>
       </c>
       <c r="E7" s="9" t="n">
-        <v>4715</v>
+        <v>3903</v>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
@@ -886,11 +886,11 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:13.691Z</t>
+          <t>2026-03-03T15:48:09.451Z</t>
         </is>
       </c>
       <c r="E8" s="9" t="n">
-        <v>386</v>
+        <v>321</v>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
@@ -917,11 +917,11 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:14.078Z</t>
+          <t>2026-03-03T15:48:09.772Z</t>
         </is>
       </c>
       <c r="E9" s="9" t="n">
-        <v>4210</v>
+        <v>3696</v>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
@@ -948,11 +948,11 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:18.288Z</t>
+          <t>2026-03-03T15:48:13.469Z</t>
         </is>
       </c>
       <c r="E10" s="9" t="n">
-        <v>2802</v>
+        <v>2772</v>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
@@ -979,11 +979,11 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:21.090Z</t>
+          <t>2026-03-03T15:48:16.240Z</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>3727</v>
+        <v>4230</v>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
@@ -1010,11 +1010,11 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:24.817Z</t>
+          <t>2026-03-03T15:48:20.470Z</t>
         </is>
       </c>
       <c r="E12" s="9" t="n">
-        <v>2708</v>
+        <v>2648</v>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
@@ -1041,11 +1041,11 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:27.525Z</t>
+          <t>2026-03-03T15:48:23.118Z</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
-        <v>4256</v>
+        <v>4113</v>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
@@ -1072,11 +1072,11 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:31.781Z</t>
+          <t>2026-03-03T15:48:27.232Z</t>
         </is>
       </c>
       <c r="E14" s="9" t="n">
-        <v>823</v>
+        <v>16168</v>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
@@ -1103,11 +1103,11 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:32.605Z</t>
+          <t>2026-03-03T15:48:43.400Z</t>
         </is>
       </c>
       <c r="E15" s="9" t="n">
-        <v>4864</v>
+        <v>15137</v>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
@@ -1134,11 +1134,11 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:37.469Z</t>
+          <t>2026-03-03T15:48:58.537Z</t>
         </is>
       </c>
       <c r="E16" s="9" t="n">
-        <v>3703</v>
+        <v>3793</v>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
@@ -1165,11 +1165,11 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:41.172Z</t>
+          <t>2026-03-03T15:49:02.331Z</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>349</v>
+        <v>333</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
@@ -1196,11 +1196,11 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:41.521Z</t>
+          <t>2026-03-03T15:49:02.665Z</t>
         </is>
       </c>
       <c r="E18" s="9" t="n">
-        <v>12947</v>
+        <v>12711</v>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
@@ -1227,11 +1227,11 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:54.469Z</t>
+          <t>2026-03-03T15:49:15.377Z</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
-        <v>4157</v>
+        <v>4206</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
@@ -1258,11 +1258,11 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:11:58.627Z</t>
+          <t>2026-03-03T15:49:19.583Z</t>
         </is>
       </c>
       <c r="E20" s="9" t="n">
-        <v>1722</v>
+        <v>1718</v>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
@@ -1289,11 +1289,11 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:00.349Z</t>
+          <t>2026-03-03T15:49:21.301Z</t>
         </is>
       </c>
       <c r="E21" s="9" t="n">
-        <v>3453</v>
+        <v>3473</v>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
@@ -1320,11 +1320,11 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:03.803Z</t>
+          <t>2026-03-03T15:49:24.774Z</t>
         </is>
       </c>
       <c r="E22" s="9" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
@@ -1351,11 +1351,11 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:04.108Z</t>
+          <t>2026-03-03T15:49:25.080Z</t>
         </is>
       </c>
       <c r="E23" s="9" t="n">
-        <v>13260</v>
+        <v>12875</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
@@ -1382,11 +1382,11 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:17.369Z</t>
+          <t>2026-03-03T15:49:37.956Z</t>
         </is>
       </c>
       <c r="E24" s="9" t="n">
-        <v>4389</v>
+        <v>4012</v>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
@@ -1413,11 +1413,11 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:21.759Z</t>
+          <t>2026-03-03T15:49:41.968Z</t>
         </is>
       </c>
       <c r="E25" s="9" t="n">
-        <v>739</v>
+        <v>16038</v>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
@@ -1444,11 +1444,11 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:22.498Z</t>
+          <t>2026-03-03T15:49:58.006Z</t>
         </is>
       </c>
       <c r="E26" s="9" t="n">
-        <v>2832</v>
+        <v>13713</v>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
@@ -1475,11 +1475,11 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:25.331Z</t>
+          <t>2026-03-03T15:50:11.719Z</t>
         </is>
       </c>
       <c r="E27" s="9" t="n">
-        <v>3433</v>
+        <v>3386</v>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
@@ -1506,11 +1506,11 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:32.102Z</t>
+          <t>2026-03-03T15:50:34.292Z</t>
         </is>
       </c>
       <c r="E28" s="9" t="n">
-        <v>577</v>
+        <v>570</v>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
@@ -1537,11 +1537,11 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:32.680Z</t>
+          <t>2026-03-03T15:50:34.862Z</t>
         </is>
       </c>
       <c r="E29" s="9" t="n">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
@@ -1568,11 +1568,11 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:33.216Z</t>
+          <t>2026-03-03T15:50:35.393Z</t>
         </is>
       </c>
       <c r="E30" s="9" t="n">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
@@ -1599,11 +1599,11 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:33.749Z</t>
+          <t>2026-03-03T15:50:35.934Z</t>
         </is>
       </c>
       <c r="E31" s="9" t="n">
-        <v>1672</v>
+        <v>1682</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -1630,11 +1630,11 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:35.422Z</t>
+          <t>2026-03-03T15:50:37.617Z</t>
         </is>
       </c>
       <c r="E32" s="9" t="n">
-        <v>890</v>
+        <v>898</v>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
@@ -1661,11 +1661,11 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:36.312Z</t>
+          <t>2026-03-03T15:50:38.516Z</t>
         </is>
       </c>
       <c r="E33" s="9" t="n">
-        <v>933</v>
+        <v>866</v>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
@@ -1692,11 +1692,11 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:37.245Z</t>
+          <t>2026-03-03T15:50:39.383Z</t>
         </is>
       </c>
       <c r="E34" s="9" t="n">
-        <v>837</v>
+        <v>829</v>
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
@@ -1723,11 +1723,11 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:38.083Z</t>
+          <t>2026-03-03T15:50:40.212Z</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
-        <v>6363</v>
+        <v>6476</v>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
@@ -1754,11 +1754,11 @@
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:44.446Z</t>
+          <t>2026-03-03T15:50:46.689Z</t>
         </is>
       </c>
       <c r="E36" s="9" t="n">
-        <v>3802</v>
+        <v>3865</v>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
@@ -1785,11 +1785,11 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:48.249Z</t>
+          <t>2026-03-03T15:50:50.555Z</t>
         </is>
       </c>
       <c r="E37" s="9" t="n">
-        <v>468</v>
+        <v>450</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
@@ -1816,11 +1816,11 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:48.717Z</t>
+          <t>2026-03-03T15:50:51.006Z</t>
         </is>
       </c>
       <c r="E38" s="9" t="n">
-        <v>454</v>
+        <v>426</v>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
@@ -1847,11 +1847,11 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:49.172Z</t>
+          <t>2026-03-03T15:50:51.432Z</t>
         </is>
       </c>
       <c r="E39" s="9" t="n">
-        <v>467</v>
+        <v>446</v>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
@@ -1878,11 +1878,11 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:49.639Z</t>
+          <t>2026-03-03T15:50:51.878Z</t>
         </is>
       </c>
       <c r="E40" s="9" t="n">
-        <v>825</v>
+        <v>839</v>
       </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
@@ -1909,11 +1909,11 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:50.465Z</t>
+          <t>2026-03-03T15:50:52.719Z</t>
         </is>
       </c>
       <c r="E41" s="9" t="n">
-        <v>5271</v>
+        <v>5272</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
@@ -1940,11 +1940,11 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:12:55.737Z</t>
+          <t>2026-03-03T15:50:57.991Z</t>
         </is>
       </c>
       <c r="E42" s="9" t="n">
-        <v>6076</v>
+        <v>6177</v>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
@@ -1971,11 +1971,11 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:13:01.814Z</t>
+          <t>2026-03-03T15:51:04.168Z</t>
         </is>
       </c>
       <c r="E43" s="9" t="n">
-        <v>2100</v>
+        <v>2038</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
@@ -2002,11 +2002,11 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:13:03.915Z</t>
+          <t>2026-03-03T15:51:06.207Z</t>
         </is>
       </c>
       <c r="E44" s="9" t="n">
-        <v>328</v>
+        <v>379</v>
       </c>
       <c r="F44" s="10" t="inlineStr">
         <is>
@@ -2033,11 +2033,11 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:13:04.244Z</t>
+          <t>2026-03-03T15:51:06.587Z</t>
         </is>
       </c>
       <c r="E45" s="9" t="n">
-        <v>2370</v>
+        <v>2379</v>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
@@ -2064,11 +2064,11 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:13:06.615Z</t>
+          <t>2026-03-03T15:51:08.966Z</t>
         </is>
       </c>
       <c r="E46" s="9" t="n">
-        <v>1350</v>
+        <v>1363</v>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
@@ -2095,11 +2095,11 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:13:07.965Z</t>
+          <t>2026-03-03T15:51:10.329Z</t>
         </is>
       </c>
       <c r="E47" s="9" t="n">
-        <v>4559</v>
+        <v>4616</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
@@ -2126,11 +2126,11 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:13:12.525Z</t>
+          <t>2026-03-03T15:51:14.945Z</t>
         </is>
       </c>
       <c r="E48" s="9" t="n">
-        <v>1579</v>
+        <v>1644</v>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
@@ -2157,11 +2157,11 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>2026-03-02T15:13:14.104Z</t>
+          <t>2026-03-03T15:51:16.589Z</t>
         </is>
       </c>
       <c r="E49" s="9" t="n">
-        <v>744</v>
+        <v>605</v>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>

</xml_diff>